<commit_message>
Rewrite organic flashcard pack from original learning points
</commit_message>
<xml_diff>
--- a/docs/flashcards/organic-names-and-formulae.xlsx
+++ b/docs/flashcards/organic-names-and-formulae.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flashcards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organic names and formulae" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Flashcards'!$A$1:$D$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Organic names and formulae'!$A$1:$D$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,10 +430,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="90" customWidth="1" min="4" max="4"/>
@@ -461,10 +461,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="75" customHeight="1">
+    <row r="2" ht="85" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>organic-names-001</t>
+          <t>organic-basics-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -474,7 +474,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds contains the –COOH group?</t>
+          <t>Which homologous series has the functional group -COOH?</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -483,10 +483,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="75" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>organic-names-002</t>
+          <t>organic-basics-002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -496,19 +496,19 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds contains an –OH group bonded to a saturated carbon atom?</t>
+          <t>What is the functional group of an alcohol?</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Alcohols.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="75" customHeight="1">
+          <t>An -OH group bonded to a saturated carbon atom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>organic-names-003</t>
+          <t>organic-basics-003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -518,19 +518,19 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds contains the –C≡N group?</t>
+          <t>Which homologous series contains a carbon-nitrogen triple bond?</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nitriles. The carbon of the –C≡N group is bonded to the rest of the molecule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="75" customHeight="1">
+          <t>Nitriles. The carbon atom of the nitrile group is bonded to the rest of the molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>organic-names-004</t>
+          <t>organic-basics-004</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds contains an –NH₂ group bonded to an alkyl group?</t>
+          <t>Which class of compounds includes molecules with an -NH2 group bonded to an alkyl group?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -549,10 +549,10 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="75" customHeight="1">
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>organic-names-005</t>
+          <t>organic-basics-005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -562,19 +562,19 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>What is the name of the –CH₃ group?</t>
+          <t>What is the name of the -CH3 substituent?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Methyl. It is an alkyl substituent, rather than a functional group.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="75" customHeight="1">
+          <t>Methyl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>organic-names-006</t>
+          <t>organic-basics-006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -584,19 +584,19 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>What is the condensed structural formula of propane?</t>
+          <t>What is the structural formula of propane?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CH₃CH₂CH₃</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="75" customHeight="1">
+          <t>CH3CH2CH3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>organic-names-007</t>
+          <t>organic-basics-007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -606,19 +606,19 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>What is the molecular formula of an acyclic hexene with one C=C bond?</t>
+          <t>What is the molecular formula of hex-1-ene?</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>C₆H₁₂</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="75" customHeight="1">
+          <t>C6H12</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="85" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>organic-names-008</t>
+          <t>organic-basics-008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -628,20 +628,19 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>What naming suffix is used for a carboxylic acid?</t>
+          <t>What suffix is used when naming a carboxylic acid?</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Suffix: -oic acid
-Example: propanoic acid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="75" customHeight="1">
+          <t>The suffix is -oic acid, as in ethanoic acid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="85" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>organic-names-009</t>
+          <t>organic-basics-009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -651,20 +650,19 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>What ending is used for the acid-derived part of an ester’s name?</t>
+          <t>What ending is used for the acid-derived part of an ester name?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Suffix: -oate
-Example: ethyl propanoate. The alkyl group bonded to oxygen is named first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="75" customHeight="1">
+          <t>The ending is -oate, as in ethyl ethanoate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="85" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>organic-names-010</t>
+          <t>organic-basics-010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -674,21 +672,20 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>What prefix and suffix can be used for an alcohol group?</t>
+          <t>What suffix and prefix are used to name an -OH group?</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Prefix: hydroxy-
-Suffix: -ol
-Use hydroxy- when the –OH group is named as a substituent because a higher-priority group supplies the suffix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="75" customHeight="1">
+          <t>The suffix is -ol, as in ethanol.
+The prefix is hydroxy- when a higher-priority functional group determines the suffix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="85" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>organic-names-011</t>
+          <t>organic-basics-011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -698,20 +695,20 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>How is an ester linkage written using R-group notation?</t>
+          <t>How can the structure of an ester be written using R groups?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>R–C(=O)–O–R′
-The carbonyl carbon is bonded directly to O–R′. The groups on the two sides need not be the same.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="75" customHeight="1">
+          <t>R-C(=O)-O-R'
+R and R' represent organic groups that may be different. In a methanoate ester, the group attached to the carbonyl carbon is H instead of R.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="85" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>organic-names-012</t>
+          <t>organic-basics-012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -721,7 +718,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds has the general structure R–O–R′?</t>
+          <t>What class of compounds has the structure R-O-R'?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -730,10 +727,10 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="75" customHeight="1">
+    <row r="14" ht="85" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>organic-names-013</t>
+          <t>organic-basics-013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -743,20 +740,20 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>How does the bonding at the carbonyl group differ in an aldehyde and a ketone?</t>
+          <t>What is the structural difference between an aldehyde and a ketone?</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Aldehyde: the carbonyl carbon is bonded to at least one hydrogen, giving a –CHO group.
-Ketone: the carbonyl carbon is bonded to two carbon atoms, giving R–C(=O)–R′.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="75" customHeight="1">
+          <t>An aldehyde has a carbonyl carbon bonded to at least one H atom: -CHO.
+A ketone has a carbonyl carbon bonded to two carbon atoms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="85" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>organic-names-014</t>
+          <t>organic-basics-014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -771,14 +768,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>A carbon–carbon double bond, C=C.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="75" customHeight="1">
+          <t>A carbon-carbon double bond, C=C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="85" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>organic-names-015</t>
+          <t>organic-basics-015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -788,7 +785,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>What type of carbon–carbon bonds are present in alkanes?</t>
+          <t>What type of carbon-carbon bonds are present in an alkane?</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -797,10 +794,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="75" customHeight="1">
+    <row r="17" ht="85" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>organic-names-016</t>
+          <t>organic-basics-016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -810,7 +807,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>What functional group is shared by aldehydes and ketones?</t>
+          <t>What group is present in both aldehydes and ketones?</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -819,10 +816,10 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="75" customHeight="1">
+    <row r="18" ht="85" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>organic-names-017</t>
+          <t>organic-basics-017</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -832,20 +829,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>What naming suffix is used for a ketone?</t>
+          <t>What suffix is used when naming a ketone?</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Suffix: -one
-Example: propanone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="75" customHeight="1">
+          <t>The suffix is -one, as in propanone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="85" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>organic-names-018</t>
+          <t>organic-basics-018</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -855,20 +851,19 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>What naming suffix is used for an aldehyde?</t>
+          <t>What suffix is used when naming an aldehyde?</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Suffix: -al
-Example: methanal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="75" customHeight="1">
+          <t>The suffix is -al, as in ethanal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="85" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>organic-names-019</t>
+          <t>organic-basics-019</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -878,20 +873,19 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>In the ester name ethyl propanoate, which part identifies the carboxylic acid from which it is derived?</t>
+          <t>What is a functional group?</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Propanoate identifies the acid-derived part; it is derived from propanoic acid.
-Ethyl identifies the alkyl group bonded to the ester oxygen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="75" customHeight="1">
+          <t>An atom or group of atoms responsible for the characteristic chemical reactions of an organic compound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="85" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>organic-names-020</t>
+          <t>organic-basics-020</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -901,19 +895,20 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>What is a functional group?</t>
+          <t>What is a homologous series?</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>An atom or group of atoms responsible for the characteristic chemical reactions of an organic compound.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="75" customHeight="1">
+          <t>A family of organic compounds with the same functional group and general formula.
+Successive members differ by CH2 and have similar chemical properties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="85" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>organic-names-021</t>
+          <t>organic-basics-021</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -923,19 +918,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>What is a homologous series?</t>
+          <t>What does a displayed formula show?</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>A family of organic compounds with the same functional group and general formula, similar chemical properties, and successive members differing by CH₂.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="75" customHeight="1">
+          <t>Every atom and every bond in a molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="85" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>organic-names-022</t>
+          <t>organic-basics-022</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -945,19 +940,20 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>What does a displayed formula show?</t>
+          <t>How do you choose the numbering direction when naming a simple branched alkane?</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>All the atoms and all the bonds between them. It does not necessarily show the molecule’s actual three-dimensional shape.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="75" customHeight="1">
+          <t>Number the parent chain to give the branches the lowest possible set of numbers.
+Compare the sets at the first point where they differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="85" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>organic-names-023</t>
+          <t>organic-basics-023</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -967,19 +963,20 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>How do you choose the numbering direction for a simple branched alkane?</t>
+          <t>How do you choose the parent chain of a simple branched alkane?</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Number the parent chain to give substituents the lowest set of locants. Compare the possible sets at the first point of difference; do not simply choose the smallest total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="75" customHeight="1">
+          <t>Choose the longest continuous carbon chain.
+The number of carbon atoms in that chain determines the stem of the name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="85" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>organic-names-024</t>
+          <t>organic-basics-024</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -989,19 +986,20 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>How is the parent chain chosen when naming a simple branched alkane?</t>
+          <t>What does R represent in an organic formula?</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Choose the longest continuous carbon chain. Its number of carbon atoms determines the stem of the name.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="75" customHeight="1">
+          <t>An unspecified organic group, usually an alkyl group.
+It is shorthand for part of the molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="85" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>organic-names-025</t>
+          <t>organic-basics-025</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1011,19 +1009,20 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>What does R represent in an organic formula?</t>
+          <t>What is an alkyl group?</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>An unspecified organic group, usually an alkyl group. R and R′ can represent different groups.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="75" customHeight="1">
+          <t>A group formed by removing one H atom from an alkane.
+For example, methane gives the methyl group, -CH3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="85" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>organic-names-026</t>
+          <t>organic-basics-026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1033,20 +1032,19 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>What is an alkyl group?</t>
+          <t>What is a haloalkane?</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>A group formed by removing one hydrogen atom from an alkane.
-Examples: methyl, –CH₃; ethyl, –CH₂CH₃.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="75" customHeight="1">
+          <t>A compound formed when one or more H atoms in an alkane are replaced by halogen atoms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="85" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>organic-names-027</t>
+          <t>organic-basics-027</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1056,19 +1054,19 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>What is a haloalkane?</t>
+          <t>Which homologous series has the functional group -C(=O)Cl?</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>A compound derived from an alkane by replacing one or more hydrogen atoms with halogen atoms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="75" customHeight="1">
+          <t>Acyl chlorides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="85" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>organic-names-028</t>
+          <t>organic-basics-028</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1078,19 +1076,20 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Which class of organic compounds contains the –C(=O)Cl group?</t>
+          <t>What is an alkane?</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Acyl chlorides. The chlorine atom is bonded directly to the carbonyl carbon.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="75" customHeight="1">
+          <t>A saturated, acyclic hydrocarbon.
+It contains only carbon and hydrogen, with single bonds only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="85" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>organic-names-029</t>
+          <t>organic-basics-029</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1100,19 +1099,19 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>What is the simplest saturated, acyclic hydrocarbon homologous series?</t>
+          <t>What ending is used when naming an acyl chloride?</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Alkanes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="75" customHeight="1">
+          <t>The ending is -oyl chloride, as in ethanoyl chloride.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="85" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>organic-names-030</t>
+          <t>organic-basics-030</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1122,20 +1121,20 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>What naming ending is used for an acyl chloride?</t>
+          <t>What is a general formula?</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Suffix: -oyl chloride
-Example: ethanoyl chloride.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="75" customHeight="1">
+          <t>An algebraic formula describing members of a homologous series.
+For example, the general formula of alkanes is CnH(2n+2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="85" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>organic-names-031</t>
+          <t>organic-basics-031</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1145,20 +1144,19 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>What is a general formula?</t>
+          <t>What is an empirical formula?</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>An algebraic formula describing members of a homologous series.
-Example: CₙH₂ₙ₊₂ for acyclic alkanes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="75" customHeight="1">
+          <t>The simplest whole-number ratio of atoms of each element in a compound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="85" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>organic-names-032</t>
+          <t>organic-basics-032</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1168,19 +1166,19 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>What is an empirical formula?</t>
+          <t>What is a molecular formula?</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>The simplest whole-number ratio of atoms of each element in a compound.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="75" customHeight="1">
+          <t>The actual number of atoms of each element in one molecule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="85" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>organic-names-033</t>
+          <t>organic-basics-033</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1190,40 +1188,18 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>What is a molecular formula?</t>
+          <t>What does a structural formula show?</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>The actual number of atoms of each element in one molecule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="75" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>organic-names-034</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>basic</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>What is a structural formula?</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>A formula showing the arrangement of atoms or groups in a molecule without displaying every bond.
-Example: CH₃CH₂CH₃ for propane.</t>
+          <t>The arrangement of atoms or groups in a molecule, without showing every bond.
+For example, CH3CH2OH is the structural formula of ethanol.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D35"/>
+  <autoFilter ref="A1:D34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align flashcard formula notation and definitions with OCR specification
</commit_message>
<xml_diff>
--- a/docs/flashcards/organic-names-and-formulae.xlsx
+++ b/docs/flashcards/organic-names-and-formulae.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
@@ -59,10 +64,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,7 +545,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Which class of compounds includes molecules with an -NH2 group bonded to an alkyl group?</t>
+          <t>Which class of compounds includes molecules with an -NH₂ group bonded to an alkyl group?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -562,7 +567,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>What is the name of the -CH3 substituent?</t>
+          <t>What is the name of the -CH₃ substituent?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -589,7 +594,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CH3CH2CH3</t>
+          <t>CH₃CH₂CH₃</t>
         </is>
       </c>
     </row>
@@ -611,7 +616,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>C6H12</t>
+          <t>C₆H₁₂</t>
         </is>
       </c>
     </row>
@@ -695,13 +700,13 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>How can the structure of an ester be written using R groups?</t>
+          <t>How is an ester written in structural formula notation using R groups?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>R-C(=O)-O-R'
-R and R' represent organic groups that may be different. In a methanoate ester, the group attached to the carbonyl carbon is H instead of R.</t>
+          <t>RCOOR′
+R and R′ represent organic groups that may be different.</t>
         </is>
       </c>
     </row>
@@ -718,7 +723,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>What class of compounds has the structure R-O-R'?</t>
+          <t>What class of compounds has the structure R–O–R′?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -900,8 +905,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>A family of organic compounds with the same functional group and general formula.
-Successive members differ by CH2 and have similar chemical properties.</t>
+          <t>A series of organic compounds having the same functional group, with each successive member differing by CH₂.</t>
         </is>
       </c>
     </row>
@@ -923,7 +927,8 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Every atom and every bond in a molecule.</t>
+          <t>The relative positioning of atoms and the bonds between them.
+Every atom and every bond is shown.</t>
         </is>
       </c>
     </row>
@@ -991,8 +996,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>An unspecified organic group, usually an alkyl group.
-It is shorthand for part of the molecule.</t>
+          <t>An alkyl group or another fragment of an organic compound that is not involved in the reaction.</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1019,7 @@
       <c r="D26" s="2" t="inlineStr">
         <is>
           <t>A group formed by removing one H atom from an alkane.
-For example, methane gives the methyl group, -CH3.</t>
+For example, methane gives the methyl group, -CH₃.</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1058,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Which homologous series has the functional group -C(=O)Cl?</t>
+          <t>Which homologous series has the functional group –COCl?</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1126,8 +1130,8 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>An algebraic formula describing members of a homologous series.
-For example, the general formula of alkanes is CnH(2n+2).</t>
+          <t>The simplest algebraic formula of a member of a homologous series.
+For alkanes: CₙH₂ₙ₊₂.</t>
         </is>
       </c>
     </row>
@@ -1193,8 +1197,8 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>The arrangement of atoms or groups in a molecule, without showing every bond.
-For example, CH3CH2OH is the structural formula of ethanol.</t>
+          <t>The minimal detail that shows the arrangement of atoms in a molecule.
+For example, CH₃CH₂OH is the structural formula of ethanol.</t>
         </is>
       </c>
     </row>

</xml_diff>